<commit_message>
add 27 crit application
</commit_message>
<xml_diff>
--- a/data27crit.xlsx
+++ b/data27crit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vincent MOUSSEAU\Dropbox\- Centrale\Pédagogie\Decision Making-ORRA\2025-26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/claravega/Documents/Cours 3A CS/SDP_3A_CS/systeme_de_decision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CD2E528-97B4-4F8D-9779-69FFE634A409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37667C0E-C7D9-3441-B289-C46E8688A3E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ED726CF5-01AA-4825-830A-635C7D11D368}"/>
+    <workbookView minimized="1" xWindow="18820" yWindow="1160" windowWidth="23260" windowHeight="13900" xr2:uid="{ED726CF5-01AA-4825-830A-635C7D11D368}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -516,29 +516,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3BB9C46-63B9-41C3-8971-88854A3C7B1E}">
   <dimension ref="A1:AB11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -621,7 +621,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -707,7 +707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -793,7 +793,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -879,7 +879,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>3</v>
       </c>
@@ -965,7 +965,7 @@
         <v>-717</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>4</v>
       </c>

</xml_diff>